<commit_message>
Remove outdated revision mistake log and add new study packs for C files, streams, preprocessor, macros, and headers. Implement scripts to generate PDF study materials with structured content and practice questions.
</commit_message>
<xml_diff>
--- a/revision-mistake-log.xlsx
+++ b/revision-mistake-log.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Mistake Log" sheetId="1" r:id="rId1"/>
-    <sheet name="Priority Redo Order" sheetId="2" r:id="rId2"/>
+    <sheet name="Tracker" sheetId="1" r:id="rId1"/>
+    <sheet name="Correct Rules" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -84,26 +84,27 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RevisionMistakeLog" displayName="RevisionMistakeLog" ref="A1:F12" totalsRowShown="0">
-  <autoFilter ref="A1:F12"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RevisionMistakeTracker" displayName="RevisionMistakeTracker" ref="A1:E18" totalsRowShown="0">
+  <autoFilter ref="A1:E18"/>
+  <tableColumns count="5">
     <tableColumn id="1" name="Topic sheet"/>
-    <tableColumn id="2" name="Question"/>
+    <tableColumn id="2" name="Question number"/>
     <tableColumn id="3" name="Topic"/>
-    <tableColumn id="4" name="My mistake"/>
-    <tableColumn id="5" name="Correct rule"/>
-    <tableColumn id="6" name="Redo prompt"/>
+    <tableColumn id="4" name="Redo prompt"/>
+    <tableColumn id="5" name="Completed"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PriorityRedoOrder" displayName="PriorityRedoOrder" ref="A1:B7" totalsRowShown="0">
-  <autoFilter ref="A1:B7"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="Priority"/>
-    <tableColumn id="2" name="Redo item"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RevisionCorrectRules" displayName="RevisionCorrectRules" ref="A1:D18" totalsRowShown="0">
+  <autoFilter ref="A1:D18"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Topic sheet"/>
+    <tableColumn id="2" name="Question number"/>
+    <tableColumn id="3" name="Topic"/>
+    <tableColumn id="4" name="Correct rule"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -116,9 +117,8 @@
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="24" customWidth="1"/>
-    <col min="4" max="4" width="42" customWidth="1"/>
-    <col min="5" max="5" width="58" customWidth="1"/>
-    <col min="6" max="6" width="48" customWidth="1"/>
+    <col min="4" max="4" width="52" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -129,7 +129,7 @@
       </c>
       <c r="B1" t="inlineStr" s="1">
         <is>
-          <t>Question</t>
+          <t>Question number</t>
         </is>
       </c>
       <c r="C1" t="inlineStr" s="1">
@@ -139,17 +139,12 @@
       </c>
       <c r="D1" t="inlineStr" s="1">
         <is>
-          <t>My mistake</t>
+          <t>Redo prompt</t>
         </is>
       </c>
       <c r="E1" t="inlineStr" s="1">
         <is>
-          <t>Correct rule</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr" s="1">
-        <is>
-          <t>Redo prompt</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -171,17 +166,12 @@
       </c>
       <c r="D2" t="inlineStr" s="2">
         <is>
-          <t>I did not realise that `x` is the integer value itself.</t>
+          <t>For `int x = 4; int *p = &amp;x;`, state only what `x` is.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr" s="2">
         <is>
-          <t>In `int x = 4; int *p = &amp;x;`, `x` is the stored integer value, `&amp;x` is its address, `p` stores that address, `*p` is the value at that address, and `&amp;p` is the address of the pointer variable.</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr" s="2">
-        <is>
-          <t>Explain `x`, `&amp;x`, `p`, `*p`, and `&amp;p` for `int x = 4; int *p = &amp;x;`.</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -203,17 +193,12 @@
       </c>
       <c r="D3" t="inlineStr" s="2">
         <is>
-          <t>I said the length was 5 but did not explain that `strlen` stops at the null terminator.</t>
+          <t>For `char s[20] = "Hello";`, explain only why `strlen(s)` is 5.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr" s="2">
         <is>
-          <t>`strlen(s)` counts characters until it reaches `'\0'`, not including the null terminator. `sizeof(s)` gives the bytes reserved for the array itself.</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr" s="2">
-        <is>
-          <t>For `char s[20] = "Hello";`, explain why `strlen(s)` is 5 and `sizeof(s)` is 20.</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -235,17 +220,12 @@
       </c>
       <c r="D4" t="inlineStr" s="2">
         <is>
-          <t>I did not mention that out-of-bounds writes can corrupt nearby data, change another variable, or cause a segmentation fault.</t>
+          <t>List three possible results of writing past the end of an array in C.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr" s="2">
         <is>
-          <t>Writing outside an array is undefined behaviour. It might appear to work, corrupt memory, change another variable, or crash with a segmentation fault.</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr" s="2">
-        <is>
-          <t>Explain why `array[15] = 999;` is unsafe when `array` has 10 elements.</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -267,17 +247,12 @@
       </c>
       <c r="D5" t="inlineStr" s="2">
         <is>
-          <t>I forgot to add the `if (a != NULL)` / `if (a == NULL)` check after `malloc`.</t>
+          <t>Write only the allocation and `NULL` check for an `int *a` array of size `n`.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr" s="2">
         <is>
-          <t>`malloc` can fail and return `NULL`. Check the pointer before writing through it. Only use the array if allocation succeeded, then `free` it afterwards.</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr" s="2">
-        <is>
-          <t>Write code that allocates `n` integers, checks for failure, fills them with `1` to `n`, prints them, and frees the memory.</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -299,17 +274,12 @@
       </c>
       <c r="D6" t="inlineStr" s="2">
         <is>
-          <t>I did not get the safe fix correct and did not mention that `p` was uninitialised.</t>
+          <t>Explain why `char *p; strcpy(p, "Hello");` is unsafe, then give one safe fix.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr" s="2">
         <is>
-          <t>`char *p;` is an uninitialised pointer. `strcpy(p, "Hello")` is unsafe because `p` does not point to valid writable memory. Fix with `char p[6];` or with `malloc(6)`, a `NULL` check, `strcpy`, and `free`.</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr" s="2">
-        <is>
-          <t>Explain the bug in `char *p; strcpy(p, "Hello");` and give two safe fixes.</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -331,17 +301,12 @@
       </c>
       <c r="D7" t="inlineStr" s="2">
         <is>
-          <t>I got the 2D dynamic array allocation and freeing completely wrong.</t>
+          <t>Write the declaration, allocation pattern, and free order for `int **X` with `R` rows and `C` columns.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr" s="2">
         <is>
-          <t>For `R` rows and `C` columns: declare `int **X`, allocate the row pointer array with `malloc(R * sizeof *X)`, allocate each row with `malloc(C * sizeof *X[r])`, then free each row before freeing `X`.</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr" s="2">
-        <is>
-          <t>Write the full allocation and free pattern for `int **X` with `R` rows and `C` columns.</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -363,17 +328,12 @@
       </c>
       <c r="D8" t="inlineStr" s="2">
         <is>
-          <t>I forgot that a value can only have one owner.</t>
+          <t>Write only the Rust ownership rule about how many owners a value can have.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr" s="2">
         <is>
-          <t>Rust ownership has three rules: each value has an owner, there can only be one owner at a time, and when the owner goes out of scope the value is dropped.</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr" s="2">
-        <is>
-          <t>Write the three Rust ownership rules and explain why the one-owner rule matters.</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -395,17 +355,12 @@
       </c>
       <c r="D9" t="inlineStr" s="2">
         <is>
-          <t>I forgot to mention that Rust prevents use-after-move.</t>
+          <t>State what Rust prevents after a `String` has been moved.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr" s="2">
         <is>
-          <t>When ownership of a non-`Copy` value such as `String` moves, the old variable becomes invalid. Rust rejects later use of that variable to prevent use-after-move bugs.</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr" s="2">
-        <is>
-          <t>Explain why `let s2 = s1; println!("{s1}");` fails when `s1` is a `String`.</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -427,17 +382,12 @@
       </c>
       <c r="D10" t="inlineStr" s="2">
         <is>
-          <t>I used `char in text` instead of `text.chars()`, and I forgot to mention that `&amp;str` reads text but can accept references and literals.</t>
+          <t>Write the loop header for iterating over characters in `text`, then say why `&amp;str` is a good read-only parameter type.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr" s="2">
         <is>
-          <t>Iterate over text with `text.chars()`. Use `&amp;str` for read-only text parameters because it borrows text and works with both `String` references and string literals.</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr" s="2">
-        <is>
-          <t>Write `fn count_vowels(text: &amp;str) -&gt; usize`, using `text.chars()`, and explain why `&amp;str` is the right parameter type.</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -459,17 +409,12 @@
       </c>
       <c r="D11" t="inlineStr" s="2">
         <is>
-          <t>I used `+=` instead of `push`.</t>
+          <t>Write the single line that appends the character `!` to a `String` called `text`.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr" s="2">
         <is>
-          <t>To add one `char` to a `String`, use `text.push('a')`. `+=` expects a string slice such as `"a"`, not a `char`.</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr" s="2">
-        <is>
-          <t>Write a function that appends `!` to a `String` through `&amp;mut String`.</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -491,17 +436,174 @@
       </c>
       <c r="D12" t="inlineStr" s="2">
         <is>
-          <t>I did not mention that a `String` owns heap-allocated text and that `&amp;str` is a borrowed slice with no ownership.</t>
+          <t>State who owns the text in `String` and who owns the text in `&amp;str`.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr" s="2">
         <is>
-          <t>`String` owns a block of heap memory containing text. `&amp;str` is a borrowed string slice: pointer plus length, with no ownership.</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr" s="2">
-        <is>
-          <t>Explain the difference between `String` and `&amp;str`, including ownership and heap memory.</t>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="54" customHeight="1">
+      <c r="A13" t="inlineStr" s="2">
+        <is>
+          <t>C Files and Streams</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr" s="2">
+        <is>
+          <t>Text vs binary streams</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr" s="2">
+        <is>
+          <t>State that text streams may have character translation, and binary streams do not.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="54" customHeight="1">
+      <c r="A14" t="inlineStr" s="2">
+        <is>
+          <t>C Files and Streams</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr" s="2">
+        <is>
+          <t>`scanf` basics</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr" s="2">
+        <is>
+          <t>State that `scanf` returns the number of items successfully assigned, and explain why it needs `&amp;k`.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="54" customHeight="1">
+      <c r="A15" t="inlineStr" s="2">
+        <is>
+          <t>C Files and Streams</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr" s="2">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr" s="2">
+        <is>
+          <t>Buffering and flushing</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr" s="2">
+        <is>
+          <t>State that output may be held in memory before it is written.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="54" customHeight="1">
+      <c r="A16" t="inlineStr" s="2">
+        <is>
+          <t>C Files and Streams</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr" s="2">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr" s="2">
+        <is>
+          <t>`ferror` vs `feof`</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr" s="2">
+        <is>
+          <t>State what kind of problem `ferror(fp)` reports.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1">
+      <c r="A17" t="inlineStr" s="2">
+        <is>
+          <t>C Files and Streams</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr" s="2">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr" s="2">
+        <is>
+          <t>`rewind` and `fseek`</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr" s="2">
+        <is>
+          <t>Write the code to reset the file to the start before moving 20 bytes from the beginning.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="54" customHeight="1">
+      <c r="A18" t="inlineStr" s="2">
+        <is>
+          <t>C Files and Streams</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr" s="2">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr" s="2">
+        <is>
+          <t>Open / write / flush / close</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr" s="2">
+        <is>
+          <t>Write the fragment with the `if (fp == NULL)` check included.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr" s="2">
+        <is>
+          <t/>
         </is>
       </c>
     </row>
@@ -517,91 +619,405 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="90" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="70" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
-          <t>Priority</t>
+          <t>Topic sheet</t>
         </is>
       </c>
       <c r="B1" t="inlineStr" s="1">
         <is>
-          <t>Redo item</t>
+          <t>Question number</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t>Correct rule</t>
         </is>
       </c>
     </row>
     <row r="2" ht="54" customHeight="1">
       <c r="A2" t="inlineStr" s="2">
         <is>
+          <t>C Pointers and Memory</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr" s="2">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr" s="2">
-        <is>
-          <t>Rust Ownership and Borrowing question 8: `String` vs `&amp;str`</t>
+      <c r="C2" t="inlineStr" s="2">
+        <is>
+          <t>Pointer basics</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr" s="2">
+        <is>
+          <t>In `int x = 4; int *p = &amp;x;`, `x` is the stored integer value.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="54" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
-          <t>2</t>
+          <t>C Pointers and Memory</t>
         </is>
       </c>
       <c r="B3" t="inlineStr" s="2">
         <is>
-          <t>Rust Ownership and Borrowing question 5: `&amp;str` parameters and `text.chars()`</t>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="2">
+        <is>
+          <t>`sizeof` vs `strlen`</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr" s="2">
+        <is>
+          <t>`strlen(s)` is 5 because it counts characters only up to the null terminator `\0`, not including it.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="54" customHeight="1">
       <c r="A4" t="inlineStr" s="2">
         <is>
-          <t>3</t>
+          <t>C Pointers and Memory</t>
         </is>
       </c>
       <c r="B4" t="inlineStr" s="2">
         <is>
-          <t>Rust Ownership and Borrowing question 1: ownership rules</t>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="2">
+        <is>
+          <t>Out-of-bounds access</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="2">
+        <is>
+          <t>Three valid results are: corrupting nearby memory, changing another variable, and crashing with a segmentation fault.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="54" customHeight="1">
       <c r="A5" t="inlineStr" s="2">
         <is>
-          <t>4</t>
+          <t>C Pointers and Memory</t>
         </is>
       </c>
       <c r="B5" t="inlineStr" s="2">
         <is>
-          <t>C Pointers and Memory question 9: dynamic 2D array</t>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="2">
+        <is>
+          <t>`malloc` safety check</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="2">
+        <is>
+          <t>Use `int *a = malloc(n * sizeof *a);` and then check `if (a == NULL)` before writing through `a`.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="54" customHeight="1">
       <c r="A6" t="inlineStr" s="2">
         <is>
-          <t>5</t>
+          <t>C Pointers and Memory</t>
         </is>
       </c>
       <c r="B6" t="inlineStr" s="2">
         <is>
-          <t>C Pointers and Memory question 8: `strcpy` into an uninitialised `char *`</t>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="2">
+        <is>
+          <t>`strcpy` into `char *`</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="2">
+        <is>
+          <t>`char *p;` is uninitialised, so it does not point to valid writable memory. A safe fix is `char p[6]; strcpy(p, "Hello");` or allocating with `malloc(6)` and then freeing it later.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="54" customHeight="1">
       <c r="A7" t="inlineStr" s="2">
         <is>
-          <t>6</t>
+          <t>C Pointers and Memory</t>
         </is>
       </c>
       <c r="B7" t="inlineStr" s="2">
         <is>
-          <t>C Pointers and Memory question 7: `malloc` with `NULL` check</t>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="2">
+        <is>
+          <t>Dynamic 2D array</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="2">
+        <is>
+          <t>Declare `int **X`; allocate `X = malloc(R * sizeof *X);`, allocate each row with `X[r] = malloc(C * sizeof *X[r]);`, then `free(X[r])` for each row before `free(X)`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="54" customHeight="1">
+      <c r="A8" t="inlineStr" s="2">
+        <is>
+          <t>Rust Ownership and Borrowing</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="2">
+        <is>
+          <t>Ownership rules</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="2">
+        <is>
+          <t>A value can only have one owner at a time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="54" customHeight="1">
+      <c r="A9" t="inlineStr" s="2">
+        <is>
+          <t>Rust Ownership and Borrowing</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="2">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="2">
+        <is>
+          <t>Move semantics</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="2">
+        <is>
+          <t>After a `String` is moved, Rust prevents use-after-move by rejecting any later use of the old variable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="54" customHeight="1">
+      <c r="A10" t="inlineStr" s="2">
+        <is>
+          <t>Rust Ownership and Borrowing</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="2">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="2">
+        <is>
+          <t>`&amp;str` parameters and iteration</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="2">
+        <is>
+          <t>Iterate with `for c in text.chars() { ... }`. `&amp;str` is a good read-only parameter type because it borrows text and accepts both `String` references and string literals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1">
+      <c r="A11" t="inlineStr" s="2">
+        <is>
+          <t>Rust Ownership and Borrowing</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="2">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="2">
+        <is>
+          <t>Modifying a `String`</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr" s="2">
+        <is>
+          <t>To add one `char` to a `String`, use `text.push('!')`. `+=` expects a string slice such as `"!"`, not a `char`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="54" customHeight="1">
+      <c r="A12" t="inlineStr" s="2">
+        <is>
+          <t>Rust Ownership and Borrowing</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="2">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="2">
+        <is>
+          <t>`String` vs `&amp;str`</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr" s="2">
+        <is>
+          <t>`String` owns the text it stores on the heap. `&amp;str` does not own the text; it is a borrowed string slice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="54" customHeight="1">
+      <c r="A13" t="inlineStr" s="2">
+        <is>
+          <t>C Files and Streams</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr" s="2">
+        <is>
+          <t>Text vs binary streams</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr" s="2">
+        <is>
+          <t>Text streams may have character translation. Binary streams do not have character translation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="54" customHeight="1">
+      <c r="A14" t="inlineStr" s="2">
+        <is>
+          <t>C Files and Streams</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr" s="2">
+        <is>
+          <t>`scanf` basics</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr" s="2">
+        <is>
+          <t>`scanf` returns the number of items successfully assigned. It needs `&amp;k` because it writes into the caller's variable, so it needs its address.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="54" customHeight="1">
+      <c r="A15" t="inlineStr" s="2">
+        <is>
+          <t>C Files and Streams</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr" s="2">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr" s="2">
+        <is>
+          <t>Buffering and flushing</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr" s="2">
+        <is>
+          <t>Output may be held in memory in a buffer before it is actually written to the file or device.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="54" customHeight="1">
+      <c r="A16" t="inlineStr" s="2">
+        <is>
+          <t>C Files and Streams</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr" s="2">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr" s="2">
+        <is>
+          <t>`ferror` vs `feof`</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr" s="2">
+        <is>
+          <t>`ferror(fp)` reports general file-operation errors on the stream. `feof(fp)` reports end-of-file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1">
+      <c r="A17" t="inlineStr" s="2">
+        <is>
+          <t>C Files and Streams</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr" s="2">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr" s="2">
+        <is>
+          <t>`rewind` and `fseek`</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr" s="2">
+        <is>
+          <t>Use `rewind(fp);` first, then `fseek(fp, 20, SEEK_SET);`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="54" customHeight="1">
+      <c r="A18" t="inlineStr" s="2">
+        <is>
+          <t>C Files and Streams</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr" s="2">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr" s="2">
+        <is>
+          <t>Open / write / flush / close</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr" s="2">
+        <is>
+          <t>Open with `fopen`, immediately check `if (fp == NULL)`, then write with `fprintf`, flush if needed, and close with `fclose`.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Rust Collections and Data Modelling study pack and update revision mistake log
</commit_message>
<xml_diff>
--- a/revision-mistake-log.xlsx
+++ b/revision-mistake-log.xlsx
@@ -84,8 +84,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RevisionMistakeTracker" displayName="RevisionMistakeTracker" ref="A1:E30" totalsRowShown="0">
-  <autoFilter ref="A1:E30"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RevisionMistakeTracker" displayName="RevisionMistakeTracker" ref="A1:E36" totalsRowShown="0">
+  <autoFilter ref="A1:E36"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Topic sheet"/>
     <tableColumn id="2" name="Question number"/>
@@ -98,8 +98,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RevisionCorrectRules" displayName="RevisionCorrectRules" ref="A1:D30" totalsRowShown="0">
-  <autoFilter ref="A1:D30"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RevisionCorrectRules" displayName="RevisionCorrectRules" ref="A1:D36" totalsRowShown="0">
+  <autoFilter ref="A1:D36"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Topic sheet"/>
     <tableColumn id="2" name="Question number"/>
@@ -931,6 +931,168 @@
         </is>
       </c>
     </row>
+    <row r="31" ht="54" customHeight="1">
+      <c r="A31" t="inlineStr" s="2">
+        <is>
+          <t>Rust Collections and Data Modelling</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr" s="2">
+        <is>
+          <t>`&amp;str` parameter calls</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr" s="2">
+        <is>
+          <t>Given `fn print_text(text: &amp;str) { println!("{text}"); }` and `let text = String::from("hello");`, write one call with a string literal and one call with the `String` value.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="54" customHeight="1">
+      <c r="A32" t="inlineStr" s="2">
+        <is>
+          <t>Rust Collections and Data Modelling</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr" s="2">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr" s="2">
+        <is>
+          <t>Modifying a `String`</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr" s="2">
+        <is>
+          <t>Starting from `let mut text = String::from("Hi");`, write code that produces exactly `Hi! there`, and identify which method takes a `char` versus a `&amp;str`.</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="54" customHeight="1">
+      <c r="A33" t="inlineStr" s="2">
+        <is>
+          <t>Rust Collections and Data Modelling</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr" s="2">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr" s="2">
+        <is>
+          <t>`Vec::get` missing case</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr" s="2">
+        <is>
+          <t>For `let v = vec![10, 20, 30];`, compare `v[10]` with `v.get(10)`. Include what happens when the index is missing and show how to handle the `get` result.</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="54" customHeight="1">
+      <c r="A34" t="inlineStr" s="2">
+        <is>
+          <t>Rust Collections and Data Modelling</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr" s="2">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr" s="2">
+        <is>
+          <t>`String` field construction</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr" s="2">
+        <is>
+          <t>Given `struct Book { title: String, pages: u32 }`, create a `Book` from the literal `"Rust"` without using a `&amp;str` where a `String` is required.</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="54" customHeight="1">
+      <c r="A35" t="inlineStr" s="2">
+        <is>
+          <t>Rust Collections and Data Modelling</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr" s="2">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr" s="2">
+        <is>
+          <t>`&amp;self` vs `&amp;mut self`</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr" s="2">
+        <is>
+          <t>In an `impl Counter`, write one method that only reads `value` using `&amp;self` and one method that changes `value` using `&amp;mut self`. Explain why the second one needs `mut`.</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="54" customHeight="1">
+      <c r="A36" t="inlineStr" s="2">
+        <is>
+          <t>Rust Collections and Data Modelling</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr" s="2">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr" s="2">
+        <is>
+          <t>`Option&lt;T&gt;` and null safety</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr" s="2">
+        <is>
+          <t>Explain why returning `Option&lt;&amp;T&gt;` from a lookup is safer than returning a possible null pointer. Mention what the caller must handle before using the value.</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -1609,6 +1771,138 @@
         </is>
       </c>
     </row>
+    <row r="31" ht="72" customHeight="1">
+      <c r="A31" t="inlineStr" s="2">
+        <is>
+          <t>Rust Collections and Data Modelling</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr" s="2">
+        <is>
+          <t>`&amp;str` parameter calls</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr" s="2">
+        <is>
+          <t>A function taking `&amp;str` can be called with a string literal directly, but a `String` value must be borrowed, for example `print_text("hello")` and `print_text(&amp;text)`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="72" customHeight="1">
+      <c r="A32" t="inlineStr" s="2">
+        <is>
+          <t>Rust Collections and Data Modelling</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr" s="2">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr" s="2">
+        <is>
+          <t>Modifying a `String`</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr" s="2">
+        <is>
+          <t>Use `text.push('!')` for a single character and `text.push_str(" there")` for a string slice. A one-line `text.push_str("! there")` also gives the same final string, but it does not demonstrate both methods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="72" customHeight="1">
+      <c r="A33" t="inlineStr" s="2">
+        <is>
+          <t>Rust Collections and Data Modelling</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr" s="2">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr" s="2">
+        <is>
+          <t>`Vec::get` missing case</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr" s="2">
+        <is>
+          <t>`v[10]` panics if index 10 is missing. `v.get(10)` returns `Option&lt;&amp;i32&gt;`, so the caller can handle `Some(value)` and `None` with `match` or `if let` before using the value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="72" customHeight="1">
+      <c r="A34" t="inlineStr" s="2">
+        <is>
+          <t>Rust Collections and Data Modelling</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr" s="2">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr" s="2">
+        <is>
+          <t>`String` field construction</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr" s="2">
+        <is>
+          <t>The field type is `String`, so a string literal must be converted with `String::from("Rust")` or `"Rust".to_string()`. Parentheses around a literal do not change its type from `&amp;str` to `String`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="72" customHeight="1">
+      <c r="A35" t="inlineStr" s="2">
+        <is>
+          <t>Rust Collections and Data Modelling</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr" s="2">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr" s="2">
+        <is>
+          <t>`&amp;self` vs `&amp;mut self`</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr" s="2">
+        <is>
+          <t>`&amp;self` is an immutable borrow and is for reading. `&amp;mut self` is a mutable borrow and is required when the method changes fields such as `self.value += 1`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="72" customHeight="1">
+      <c r="A36" t="inlineStr" s="2">
+        <is>
+          <t>Rust Collections and Data Modelling</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr" s="2">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr" s="2">
+        <is>
+          <t>`Option&lt;T&gt;` and null safety</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr" s="2">
+        <is>
+          <t>`Option&lt;T&gt;` makes absence explicit as `None`. The caller must handle `Some` and `None`, so there is no chance of accidentally dereferencing a null pointer before checking whether a value exists.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Add C function pointers and callbacks study pack
- Created a new Python script to generate a PDF study pack on C function pointers and callbacks.
- Added a PDF file containing detailed explanations, code examples, and practice questions related to function pointers and callbacks in C.
- Included a compiled Python bytecode file for the new script.
</commit_message>
<xml_diff>
--- a/revision-mistake-log.xlsx
+++ b/revision-mistake-log.xlsx
@@ -84,8 +84,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RevisionMistakeTracker" displayName="RevisionMistakeTracker" ref="A1:E36" totalsRowShown="0">
-  <autoFilter ref="A1:E36"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RevisionMistakeTracker" displayName="RevisionMistakeTracker" ref="A1:E41" totalsRowShown="0">
+  <autoFilter ref="A1:E41"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Topic sheet"/>
     <tableColumn id="2" name="Question number"/>
@@ -98,8 +98,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RevisionCorrectRules" displayName="RevisionCorrectRules" ref="A1:D36" totalsRowShown="0">
-  <autoFilter ref="A1:D36"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RevisionCorrectRules" displayName="RevisionCorrectRules" ref="A1:D41" totalsRowShown="0">
+  <autoFilter ref="A1:D41"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Topic sheet"/>
     <tableColumn id="2" name="Question number"/>
@@ -166,12 +166,12 @@
       </c>
       <c r="D2" t="inlineStr" s="2">
         <is>
-          <t>Given `int x = 4; int *p = &amp;x; *p += 3; int y = *p;`, work out `x` and `y`, then identify which expression is the address.</t>
+          <t>Given `int x = 4; int *p` pointing at `x`; then `*p += 3; int y = *p;`, work out `x` and `y`, then identify which expression is the address.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -360,7 +360,7 @@
       </c>
       <c r="E9" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -377,17 +377,17 @@
       </c>
       <c r="C10" t="inlineStr" s="2">
         <is>
-          <t>`&amp;str` parameters and iteration</t>
+          <t>Borrowed string-slice parameters and iteration</t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="2">
         <is>
-          <t>Write `fn count_a(text: &amp;str) -&gt; usize` so it counts `a` characters, using the right string iteration method.</t>
+          <t>Write a `count_a` function that borrows a string slice and returns `usize`, so it counts `a` characters using the right string iteration method.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -431,7 +431,7 @@
       </c>
       <c r="C12" t="inlineStr" s="2">
         <is>
-          <t>`String` vs `&amp;str`</t>
+          <t>`String` vs borrowed string slices</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="2">
@@ -468,7 +468,7 @@
       </c>
       <c r="E13" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -490,12 +490,12 @@
       </c>
       <c r="D14" t="inlineStr" s="2">
         <is>
-          <t>For `int k = 99; int rc = scanf("%d", &amp;k);`, handle the case where the user types `abc` instead of a number.</t>
+          <t>For `int k = 99; int rc = scanf("%d", address of k);`, handle the case where the user types `abc` instead of a number.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -522,7 +522,7 @@
       </c>
       <c r="E15" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -549,7 +549,7 @@
       </c>
       <c r="E16" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
       </c>
       <c r="E17" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -603,7 +603,7 @@
       </c>
       <c r="E18" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="E20" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="E21" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="E22" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -738,7 +738,7 @@
       </c>
       <c r="E23" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -765,7 +765,7 @@
       </c>
       <c r="E24" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="D27" t="inlineStr" s="2">
         <is>
-          <t>Given `fn parse_num(text: &amp;str) -&gt; i32 { let n = text.parse::&lt;i32&gt;()?; n }`, explain why this cannot compile and fix the return type.</t>
+          <t>Given a `parse_num` function that borrows a string slice, parses an `i32` with `?`, and returns plain `i32`, explain why this cannot compile and fix the return type.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr" s="2">
@@ -873,7 +873,7 @@
       </c>
       <c r="E28" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -900,7 +900,7 @@
       </c>
       <c r="E29" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -944,12 +944,12 @@
       </c>
       <c r="C31" t="inlineStr" s="2">
         <is>
-          <t>`&amp;str` parameter calls</t>
+          <t>Borrowed string-slice parameter calls</t>
         </is>
       </c>
       <c r="D31" t="inlineStr" s="2">
         <is>
-          <t>Given `fn print_text(text: &amp;str) { println!("{text}"); }` and `let text = String::from("hello");`, write one call with a string literal and one call with the `String` value.</t>
+          <t>Given a `print_text` function that borrows a string slice and `let text = String::from("hello");`, write one call with a string literal and one call with the `String` value.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr" s="2">
@@ -976,7 +976,7 @@
       </c>
       <c r="D32" t="inlineStr" s="2">
         <is>
-          <t>Starting from `let mut text = String::from("Hi");`, write code that produces exactly `Hi! there`, and identify which method takes a `char` versus a `&amp;str`.</t>
+          <t>Starting from `let mut text = String::from("Hi");`, write code that produces exactly `Hi! there`, and identify which method takes a `char` versus a borrowed string slice.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr" s="2">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="D34" t="inlineStr" s="2">
         <is>
-          <t>Given `struct Book { title: String, pages: u32 }`, create a `Book` from the literal `"Rust"` without using a `&amp;str` where a `String` is required.</t>
+          <t>Given `struct Book { title: String, pages: u32 }`, create a `Book` from the literal `"Rust"` without using a borrowed string slice where a `String` is required.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr" s="2">
@@ -1052,12 +1052,12 @@
       </c>
       <c r="C35" t="inlineStr" s="2">
         <is>
-          <t>`&amp;self` vs `&amp;mut self`</t>
+          <t>Immutable vs mutable self borrows</t>
         </is>
       </c>
       <c r="D35" t="inlineStr" s="2">
         <is>
-          <t>In an `impl Counter`, write one method that only reads `value` using `&amp;self` and one method that changes `value` using `&amp;mut self`. Explain why the second one needs `mut`.</t>
+          <t>In an `impl Counter`, write one method that only reads `value` using an immutable self borrow and one method that changes `value` using a mutable self borrow. Explain why the second one needs `mut`.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr" s="2">
@@ -1084,10 +1084,145 @@
       </c>
       <c r="D36" t="inlineStr" s="2">
         <is>
-          <t>Explain why returning `Option&lt;&amp;T&gt;` from a lookup is safer than returning a possible null pointer. Mention what the caller must handle before using the value.</t>
+          <t>Explain why returning `Option` containing a borrowed value from a lookup is safer than returning a possible null pointer. Mention what the caller must handle before using the value.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="54" customHeight="1">
+      <c r="A37" t="inlineStr" s="2">
+        <is>
+          <t>C Function Pointers and Callbacks</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr" s="2">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr" s="2">
+        <is>
+          <t>Callback received by `apply`</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr" s="2">
+        <is>
+          <t>Complete `int apply(int a, int b, int (*fn)(int, int)) { return _____; }`, then trace what happens when it is called as `apply(1, 3, Plus)`.</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="54" customHeight="1">
+      <c r="A38" t="inlineStr" s="2">
+        <is>
+          <t>C Function Pointers and Callbacks</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr" s="2">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr" s="2">
+        <is>
+          <t>`qsort` arguments</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr" s="2">
+        <is>
+          <t>Complete the call that sorts `int values[] = {3, 1, 2};` using `compare_ints`: `qsort(_____, _____, _____, _____);`.</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="54" customHeight="1">
+      <c r="A39" t="inlineStr" s="2">
+        <is>
+          <t>C Function Pointers and Callbacks</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr" s="2">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr" s="2">
+        <is>
+          <t>Integer comparator steps</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr" s="2">
+        <is>
+          <t>Fill in the body of `int compare_ints(const void *p, const void *q)` so it works correctly with `qsort` on an integer array.</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="54" customHeight="1">
+      <c r="A40" t="inlineStr" s="2">
+        <is>
+          <t>C Function Pointers and Callbacks</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr" s="2">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr" s="2">
+        <is>
+          <t>`const void *` comparator parameters</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr" s="2">
+        <is>
+          <t>`qsort` rejects `int compare_ints(int *a, int *b)`. Fix the signature and explain why the fixed version matches `qsort`.</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="54" customHeight="1">
+      <c r="A41" t="inlineStr" s="2">
+        <is>
+          <t>C Function Pointers and Callbacks</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr" s="2">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr" s="2">
+        <is>
+          <t>Pointer arithmetic with `char *`</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr" s="2">
+        <is>
+          <t>In generic array code with `void *array` and `size_t width`, write the expression for the address of element `i` after converting the base pointer to `char *`.</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr" s="2">
         <is>
           <t/>
         </is>
@@ -1305,7 +1440,7 @@
       </c>
       <c r="D9" t="inlineStr" s="2">
         <is>
-          <t>Change the function to borrow instead of take ownership. Prefer a borrowed string-slice parameter; call it with a borrow of `name`, then `name` can still be printed.</t>
+          <t>Change the function to borrow a string slice instead of taking ownership, then call it with a borrow of `name`. A borrow does not move `name`, so it can still be printed.</t>
         </is>
       </c>
     </row>
@@ -1322,7 +1457,7 @@
       </c>
       <c r="C10" t="inlineStr" s="2">
         <is>
-          <t>`&amp;str` parameters and iteration</t>
+          <t>Borrowed string-slice parameters and iteration</t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="2">
@@ -1366,12 +1501,12 @@
       </c>
       <c r="C12" t="inlineStr" s="2">
         <is>
-          <t>`String` vs `&amp;str`</t>
+          <t>`String` vs borrowed string slices</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="2">
         <is>
-          <t>Use a string slice for read-only text. A string literal can be passed directly, and a `String` value can be passed by borrowing it.</t>
+          <t>Use a borrowed string-slice parameter for read-only text. A string literal can be passed directly, and a `String` value can be passed by borrowing it.</t>
         </is>
       </c>
     </row>
@@ -1635,7 +1770,7 @@
       </c>
       <c r="D24" t="inlineStr" s="2">
         <is>
-          <t>Use the class template with its type parameter, not plain `Stack`. For the outside `pop` definition: write the template line for `T`, then return `T`, then define `pop` inside Stack of T.</t>
+          <t>The completed header is `template&lt;typename T&gt; T Stack&lt;T&gt;::pop()`. The `Stack&lt;T&gt;` part is needed because `pop` belongs to the class template instantiated with `T`.</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1814,7 @@
       </c>
       <c r="D26" t="inlineStr" s="2">
         <is>
-          <t>Iterator pattern: start with `auto it = v.begin()`, continue while `it != v.end()`, increment with `it++`, and print the current value with `*it`.</t>
+          <t>Use `for (auto it = v.begin(); it != v.end(); ++it) { std::cout &lt;&lt; *it; }`. The iterator points at each element, and `*it` reads the current value.</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1836,7 @@
       </c>
       <c r="D27" t="inlineStr" s="2">
         <is>
-          <t>`?` can stop the function and return the error early. That means the function must return a compatible `Result`, not plain `i32`.</t>
+          <t>`?` can return the parse error early, so the function must return a compatible `Result`, such as a result containing `i32` on success and `std::num::ParseIntError` on failure, then return `Ok(n)`.</t>
         </is>
       </c>
     </row>
@@ -1723,7 +1858,7 @@
       </c>
       <c r="D28" t="inlineStr" s="2">
         <is>
-          <t>Parse the quantity. If parsing succeeds, use the number. If parsing fails, return `Err("bad quantity".to_string())`; this can be written with `map_err` or `match`.</t>
+          <t>Use `let quantity = parts[1].trim().parse::&lt;u32&gt;().map_err(|_| "bad quantity".to_string())?;` so a parse failure becomes the requested `Err` message.</t>
         </is>
       </c>
     </row>
@@ -1767,7 +1902,7 @@
       </c>
       <c r="D30" t="inlineStr" s="2">
         <is>
-          <t>Make `main` return a `Result` with an error box so different error types can be propagated. Finish successful execution with `Ok(())`.</t>
+          <t>Use `fn main() -&gt; Result&lt;(), Box&lt;dyn std::error::Error&gt;&gt;` so file-read and parse errors can be propagated with `?`. Finish successful execution with `Ok(())`.</t>
         </is>
       </c>
     </row>
@@ -1784,12 +1919,12 @@
       </c>
       <c r="C31" t="inlineStr" s="2">
         <is>
-          <t>`&amp;str` parameter calls</t>
+          <t>Borrowed string-slice parameter calls</t>
         </is>
       </c>
       <c r="D31" t="inlineStr" s="2">
         <is>
-          <t>A function taking `&amp;str` can be called with a string literal directly, but a `String` value must be borrowed, for example `print_text("hello")` and `print_text(&amp;text)`.</t>
+          <t>A function taking a borrowed string slice can be called with a string literal directly. A `String` value must be borrowed, so call with the string literal first and then call again by borrowing `text`.</t>
         </is>
       </c>
     </row>
@@ -1833,7 +1968,7 @@
       </c>
       <c r="D33" t="inlineStr" s="2">
         <is>
-          <t>`v[10]` panics if index 10 is missing. `v.get(10)` returns `Option&lt;&amp;i32&gt;`, so the caller can handle `Some(value)` and `None` with `match` or `if let` before using the value.</t>
+          <t>`v[10]` panics if index 10 is missing. `v.get(10)` returns an `Option` containing a possible borrowed value, so the caller can handle `Some(value)` and `None` with `match` or `if let`.</t>
         </is>
       </c>
     </row>
@@ -1855,7 +1990,7 @@
       </c>
       <c r="D34" t="inlineStr" s="2">
         <is>
-          <t>The field type is `String`, so a string literal must be converted with `String::from("Rust")` or `"Rust".to_string()`. Parentheses around a literal do not change its type from `&amp;str` to `String`.</t>
+          <t>The field type is `String`, so a string literal must be converted with `String::from("Rust")` or `"Rust".to_string()`. Parentheses around a literal do not change it from a borrowed string slice to `String`.</t>
         </is>
       </c>
     </row>
@@ -1872,12 +2007,12 @@
       </c>
       <c r="C35" t="inlineStr" s="2">
         <is>
-          <t>`&amp;self` vs `&amp;mut self`</t>
+          <t>Immutable vs mutable self borrows</t>
         </is>
       </c>
       <c r="D35" t="inlineStr" s="2">
         <is>
-          <t>`&amp;self` is an immutable borrow and is for reading. `&amp;mut self` is a mutable borrow and is required when the method changes fields such as `self.value += 1`.</t>
+          <t>An immutable self borrow is for reading. A mutable self borrow is required when the method changes fields such as `self.value += 1`.</t>
         </is>
       </c>
     </row>
@@ -1899,7 +2034,117 @@
       </c>
       <c r="D36" t="inlineStr" s="2">
         <is>
-          <t>`Option&lt;T&gt;` makes absence explicit as `None`. The caller must handle `Some` and `None`, so there is no chance of accidentally dereferencing a null pointer before checking whether a value exists.</t>
+          <t>Returning an `Option` containing a borrowed value makes absence explicit as `None`. The caller must handle `Some` and `None`, so there is no chance of accidentally dereferencing a null pointer before checking whether a value exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="72" customHeight="1">
+      <c r="A37" t="inlineStr" s="2">
+        <is>
+          <t>C Function Pointers and Callbacks</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr" s="2">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr" s="2">
+        <is>
+          <t>Callback received by `apply`</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr" s="2">
+        <is>
+          <t>The callback is `Plus`. `apply` receives `Plus` through its function pointer parameter, then calls that pointer to decide what operation to perform.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="72" customHeight="1">
+      <c r="A38" t="inlineStr" s="2">
+        <is>
+          <t>C Function Pointers and Callbacks</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr" s="2">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr" s="2">
+        <is>
+          <t>`qsort` arguments</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr" s="2">
+        <is>
+          <t>`qsort` receives the base pointer, number of elements, size of each element in bytes, and comparator callback. For `int values[] = {3, 1, 2};`, use `values`, 3, `sizeof values[0]`, and `compare_ints`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="72" customHeight="1">
+      <c r="A39" t="inlineStr" s="2">
+        <is>
+          <t>C Function Pointers and Callbacks</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr" s="2">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr" s="2">
+        <is>
+          <t>Integer comparator steps</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr" s="2">
+        <is>
+          <t>An integer comparator receives two `const void *` pointers, treats them as `const int *`, compares the pointed-to integer values, and returns negative, zero, or positive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="72" customHeight="1">
+      <c r="A40" t="inlineStr" s="2">
+        <is>
+          <t>C Function Pointers and Callbacks</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr" s="2">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr" s="2">
+        <is>
+          <t>`const void *` comparator parameters</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr" s="2">
+        <is>
+          <t>`qsort` is generic, so the comparator receives pointers to elements of unknown type. `const` means those pointed-to elements are read-only inside the comparator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="72" customHeight="1">
+      <c r="A41" t="inlineStr" s="2">
+        <is>
+          <t>C Function Pointers and Callbacks</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr" s="2">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr" s="2">
+        <is>
+          <t>Pointer arithmetic with `char *`</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr" s="2">
+        <is>
+          <t>Pointer arithmetic moves by the size of the pointed-to type. Generic array code uses `char *` because one step is one byte, so byte offsets such as `i * width` can locate element `i`.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add C++ Operator Overloading and Rust Generics & Traits Study Packs
- Created a C++ Operator Overloading study pack PDF and corresponding Python script to generate it.
- Added Rust Generics and Traits study pack PDF and Python script for generation.
- Included detailed explanations, code examples, practice questions, and mark schemes in both study packs.
- Generated binary files for compiled Python scripts in the __pycache__ directory.
</commit_message>
<xml_diff>
--- a/revision-mistake-log.xlsx
+++ b/revision-mistake-log.xlsx
@@ -84,8 +84,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RevisionMistakeTracker" displayName="RevisionMistakeTracker" ref="A1:E41" totalsRowShown="0">
-  <autoFilter ref="A1:E41"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RevisionMistakeTracker" displayName="RevisionMistakeTracker" ref="A1:E49" totalsRowShown="0">
+  <autoFilter ref="A1:E49"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Topic sheet"/>
     <tableColumn id="2" name="Question number"/>
@@ -98,8 +98,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RevisionCorrectRules" displayName="RevisionCorrectRules" ref="A1:D41" totalsRowShown="0">
-  <autoFilter ref="A1:D41"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RevisionCorrectRules" displayName="RevisionCorrectRules" ref="A1:D49" totalsRowShown="0">
+  <autoFilter ref="A1:D49"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Topic sheet"/>
     <tableColumn id="2" name="Question number"/>
@@ -630,7 +630,7 @@
       </c>
       <c r="E19" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="E25" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -819,7 +819,7 @@
       </c>
       <c r="E26" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="E27" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
       </c>
       <c r="E30" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -954,7 +954,7 @@
       </c>
       <c r="E31" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
       </c>
       <c r="E32" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="E33" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1035,7 +1035,7 @@
       </c>
       <c r="E34" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="E35" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="E36" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1223,6 +1223,222 @@
         </is>
       </c>
       <c r="E41" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="54" customHeight="1">
+      <c r="A42" t="inlineStr" s="2">
+        <is>
+          <t>C++ Operator Overloading</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr" s="2">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr" s="2">
+        <is>
+          <t>`MyInteger + int` member overload</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr" s="2">
+        <is>
+          <t>Given `class MyInteger { int i; public: MyInteger(int value) : i(value) {} /* missing */ };`, write the member overload that makes `MyInteger a(4); int x = a + 6;` set `x` to 10.</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="54" customHeight="1">
+      <c r="A43" t="inlineStr" s="2">
+        <is>
+          <t>C++ Operator Overloading</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr" s="2">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr" s="2">
+        <is>
+          <t>Legal and sensible overloads</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr" s="2">
+        <is>
+          <t>For `Point`, judge these attempted meanings: `Point + Point`, `int + int`, `sizeof point`, and `point.x`. Mark each as legal or illegal to overload, then choose whether the legal one is sensible.</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="54" customHeight="1">
+      <c r="A44" t="inlineStr" s="2">
+        <is>
+          <t>C++ Operator Overloading</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr" s="2">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr" s="2">
+        <is>
+          <t>`operator[]` reference return</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr" s="2">
+        <is>
+          <t>Complete an array class subscript operator so `arr[2] = 99;` changes the stored element. The body should return the element itself, not its address.</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="54" customHeight="1">
+      <c r="A45" t="inlineStr" s="2">
+        <is>
+          <t>Rust Generics and Traits</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr" s="2">
+        <is>
+          <t>Generic `Point` method</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr" s="2">
+        <is>
+          <t>Given a generic `Point` with fields `x` and `y`, complete the `impl` block so method `x` borrows the object and returns a borrow of the `x` field.</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="54" customHeight="1">
+      <c r="A46" t="inlineStr" s="2">
+        <is>
+          <t>Rust Generics and Traits</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr" s="2">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr" s="2">
+        <is>
+          <t>Borrowed generic `Area` parameter</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr" s="2">
+        <is>
+          <t>Fix a broken free function that tries to use `self.area()` outside an `impl` block, so it prints the area of any borrowed shape that implements `Area`.</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="54" customHeight="1">
+      <c r="A47" t="inlineStr" s="2">
+        <is>
+          <t>Rust Generics and Traits</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr" s="2">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr" s="2">
+        <is>
+          <t>`show_larger` display bound</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr" s="2">
+        <is>
+          <t>Fix the signature of `show_larger` when its body compares two values and then prints the winning value with normal braces.</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="54" customHeight="1">
+      <c r="A48" t="inlineStr" s="2">
+        <is>
+          <t>Rust Generics and Traits</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr" s="2">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr" s="2">
+        <is>
+          <t>`derive` attribute syntax</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr" s="2">
+        <is>
+          <t>Repair the derive line for a custom struct used with `assert_eq!` and debug printing: `#derive Debug, PartialEq`.</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="54" customHeight="1">
+      <c r="A49" t="inlineStr" s="2">
+        <is>
+          <t>Rust Generics and Traits</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr" s="2">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr" s="2">
+        <is>
+          <t>`HashMap` key derives</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr" s="2">
+        <is>
+          <t>A custom `Team` value is used as a key in a `HashMap`. Add the derives needed so insertion and lookup by key compile.</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr" s="2">
         <is>
           <t/>
         </is>
@@ -2148,6 +2364,182 @@
         </is>
       </c>
     </row>
+    <row r="42" ht="72" customHeight="1">
+      <c r="A42" t="inlineStr" s="2">
+        <is>
+          <t>C++ Operator Overloading</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr" s="2">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr" s="2">
+        <is>
+          <t>`MyInteger + int` member overload</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr" s="2">
+        <is>
+          <t>Use a member overload that takes an integer value and returns `i + value`. This handles `a + 6` because the left operand is the `MyInteger` object.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="72" customHeight="1">
+      <c r="A43" t="inlineStr" s="2">
+        <is>
+          <t>C++ Operator Overloading</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr" s="2">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr" s="2">
+        <is>
+          <t>Legal and sensible overloads</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr" s="2">
+        <is>
+          <t>`Point + Point` can be overloaded because a class type is involved, if point addition is meaningful. `int + int` cannot be changed, and `sizeof` and `.` cannot be overloaded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="72" customHeight="1">
+      <c r="A44" t="inlineStr" s="2">
+        <is>
+          <t>C++ Operator Overloading</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr" s="2">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr" s="2">
+        <is>
+          <t>`operator[]` reference return</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr" s="2">
+        <is>
+          <t>The subscript operator should return a reference to the stored element. Return `data[index]`, not the address of `data[index]`, so assignment through `arr[2]` updates the array element.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="72" customHeight="1">
+      <c r="A45" t="inlineStr" s="2">
+        <is>
+          <t>Rust Generics and Traits</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr" s="2">
+        <is>
+          <t>Generic `Point` method</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr" s="2">
+        <is>
+          <t>The `impl` block must introduce the generic type parameter, and the method should borrow `self` and return a borrow of `self.x`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="72" customHeight="1">
+      <c r="A46" t="inlineStr" s="2">
+        <is>
+          <t>Rust Generics and Traits</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr" s="2">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr" s="2">
+        <is>
+          <t>Borrowed generic `Area` parameter</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr" s="2">
+        <is>
+          <t>This should be a free function with a borrowed parameter such as `shape`, not a method using `self`. The generic type must be constrained by the `Area` trait before calling `shape.area()`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="72" customHeight="1">
+      <c r="A47" t="inlineStr" s="2">
+        <is>
+          <t>Rust Generics and Traits</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr" s="2">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr" s="2">
+        <is>
+          <t>`show_larger` display bound</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr" s="2">
+        <is>
+          <t>Comparison needs `PartialOrd`, and printing with normal braces needs `std::fmt::Display`; the generic bound needs both.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="72" customHeight="1">
+      <c r="A48" t="inlineStr" s="2">
+        <is>
+          <t>Rust Generics and Traits</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr" s="2">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr" s="2">
+        <is>
+          <t>`derive` attribute syntax</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr" s="2">
+        <is>
+          <t>The derive attribute needs square brackets and parentheses: `#[derive(Debug, PartialEq)]`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="72" customHeight="1">
+      <c r="A49" t="inlineStr" s="2">
+        <is>
+          <t>Rust Generics and Traits</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr" s="2">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr" s="2">
+        <is>
+          <t>`HashMap` key derives</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr" s="2">
+        <is>
+          <t>A `HashMap` key needs hashing and reliable equality. Usual derives are `Debug`, `Clone`, `PartialEq`, `Eq`, and `Hash`; the key requirements are `PartialEq`, `Eq`, and `Hash`.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Add study packs for C command-line arguments and Rust concurrency/parallelism
- Created `make_c_command_line_arguments_study_pack.py` to generate a PDF study pack covering key concepts of command-line arguments in C, including argc, argv, quoting, and safe conversion checks.
- Created `make_rust_concurrency_parallelism_study_pack.py` to generate a PDF study pack on Rust concurrency and parallelism, detailing threads, move closures, channels, Arc, Mutex, and parallel aggregation patterns.
- Generated the corresponding PDF files for both study packs.
</commit_message>
<xml_diff>
--- a/revision-mistake-log.xlsx
+++ b/revision-mistake-log.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="164">
   <si>
     <t>Topic sheet</t>
   </si>
@@ -491,6 +491,21 @@
   </si>
   <si>
     <t>Given `auto x = 10; x = "hello";`, explain the compile error and what `auto` did, without describing it as dynamic typing.</t>
+  </si>
+  <si>
+    <t>C Command-line Arguments</t>
+  </si>
+  <si>
+    <t>`atoi` invalid input vs zero</t>
+  </si>
+  <si>
+    <t>For `int n = atoi(argv[1]);`, compare `argv[1]` values `"abc"` and `"0"`: state what each returns and why the return value alone cannot prove the input was valid.</t>
+  </si>
+  <si>
+    <t>`strtol` no digits consumed</t>
+  </si>
+  <si>
+    <t>For `char *end; long n = strtol(text, &amp;end, 10);`, explain what `end == text` means for `text = "abc"`, then say what `*end` should be after a clean full-number parse.</t>
   </si>
 </sst>
 </file>
@@ -515,7 +530,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -572,7 +587,7 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+      <alignment horizontal="general" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -589,8 +604,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E62" displayName="RevisionMistakeTracker" name="RevisionMistakeTracker" id="1" totalsRowShown="0">
-  <autoFilter ref="A1:E62"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E64" displayName="RevisionMistakeTracker" name="RevisionMistakeTracker" id="1" totalsRowShown="0">
+  <autoFilter ref="A1:E64"/>
   <tableColumns count="5">
     <tableColumn name="Topic sheet" id="1"/>
     <tableColumn name="Question number" id="2"/>
@@ -890,7 +905,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="4" width="28.005" customWidth="1" bestFit="1"/>
@@ -1525,7 +1540,9 @@
       <c r="D37" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="E37" s="3"/>
+      <c r="E37" s="3" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="54" customFormat="1" s="1">
       <c r="A38" s="3" t="s">
@@ -1659,9 +1676,11 @@
       <c r="D45" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="E45" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="33.75" customFormat="1" s="1">
+      <c r="E45" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="54" customFormat="1" s="1">
       <c r="A46" s="3" t="s">
         <v>117</v>
       </c>
@@ -1674,9 +1693,11 @@
       <c r="D46" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="E46" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="33.75" customFormat="1" s="1">
+      <c r="E46" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="54" customFormat="1" s="1">
       <c r="A47" s="3" t="s">
         <v>117</v>
       </c>
@@ -1689,9 +1710,11 @@
       <c r="D47" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="E47" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="33.75" customFormat="1" s="1">
+      <c r="E47" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="32.25" customFormat="1" s="1">
       <c r="A48" s="3" t="s">
         <v>117</v>
       </c>
@@ -1708,7 +1731,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="33.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="32.25" customFormat="1" s="1">
       <c r="A49" s="3" t="s">
         <v>117</v>
       </c>
@@ -1725,7 +1748,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="47.25" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="45.75" customFormat="1" s="1">
       <c r="A50" s="3" t="s">
         <v>128</v>
       </c>
@@ -1742,7 +1765,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="33.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="32.25" customFormat="1" s="1">
       <c r="A51" s="3" t="s">
         <v>128</v>
       </c>
@@ -1759,7 +1782,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="47.25" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="45.75" customFormat="1" s="1">
       <c r="A52" s="3" t="s">
         <v>128</v>
       </c>
@@ -1772,9 +1795,11 @@
       <c r="D52" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="E52" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="47.25" customFormat="1" s="1">
+      <c r="E52" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="45.75" customFormat="1" s="1">
       <c r="A53" s="3" t="s">
         <v>135</v>
       </c>
@@ -1791,7 +1816,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="47.25" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="45.75" customFormat="1" s="1">
       <c r="A54" s="3" t="s">
         <v>135</v>
       </c>
@@ -1804,9 +1829,11 @@
       <c r="D54" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="E54" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="47.25" customFormat="1" s="1">
+      <c r="E54" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="45.75" customFormat="1" s="1">
       <c r="A55" s="3" t="s">
         <v>135</v>
       </c>
@@ -1823,7 +1850,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="33.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="32.25" customFormat="1" s="1">
       <c r="A56" s="3" t="s">
         <v>142</v>
       </c>
@@ -1840,7 +1867,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="33.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="32.25" customFormat="1" s="1">
       <c r="A57" s="3" t="s">
         <v>142</v>
       </c>
@@ -1857,7 +1884,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="47.25" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="45.75" customFormat="1" s="1">
       <c r="A58" s="3" t="s">
         <v>147</v>
       </c>
@@ -1870,9 +1897,11 @@
       <c r="D58" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="E58" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="47.25" customFormat="1" s="1">
+      <c r="E58" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="45.75" customFormat="1" s="1">
       <c r="A59" s="3" t="s">
         <v>147</v>
       </c>
@@ -1885,9 +1914,11 @@
       <c r="D59" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="E59" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="47.25" customFormat="1" s="1">
+      <c r="E59" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="45.75" customFormat="1" s="1">
       <c r="A60" s="3" t="s">
         <v>152</v>
       </c>
@@ -1902,7 +1933,7 @@
       </c>
       <c r="E60" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="33.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="54" customFormat="1" s="1">
       <c r="A61" s="3" t="s">
         <v>152</v>
       </c>
@@ -1915,9 +1946,11 @@
       <c r="D61" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="E61" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="33.75" customFormat="1" s="1">
+      <c r="E61" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="54" customFormat="1" s="1">
       <c r="A62" s="3" t="s">
         <v>152</v>
       </c>
@@ -1931,6 +1964,36 @@
         <v>158</v>
       </c>
       <c r="E62" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="54" customFormat="1" s="1">
+      <c r="A63" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="E63" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="54" customFormat="1" s="1">
+      <c r="A64" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E64" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add C++ Error Handling and Lambdas Study Pack and Rust Crash-course Basics Study Pack
- Updated revision-rag-topic-list.md to include new study packs for C++ error handling and Rust crash-course basics.
- Added cpp-error-handling-lambdas-study-pack.pdf containing focused revision material on exception handling and lambda syntax in C++.
- Created make_cpp_error_handling_lambdas_study_pack.py to generate the C++ study pack PDF.
- Added rust-crash-course-basics-study-pack.pdf with essential Rust concepts including variables, types, and error handling.
- Implemented make_rust_crash_course_basics_study_pack.py to generate the Rust study pack PDF.
</commit_message>
<xml_diff>
--- a/revision-mistake-log.xlsx
+++ b/revision-mistake-log.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="176">
   <si>
     <t>Topic sheet</t>
   </si>
@@ -506,6 +506,42 @@
   </si>
   <si>
     <t>For `char *end; long n = strtol(text, &amp;end, 10);`, explain what `end == text` means for `text = "abc"`, then say what `*end` should be after a clean full-number parse.</t>
+  </si>
+  <si>
+    <t>Rust Concurrency and Parallelism</t>
+  </si>
+  <si>
+    <t>Spawned thread lifetime and `move`</t>
+  </si>
+  <si>
+    <t>In `fn start() { let text = String::from("hi"); thread::spawn(|| println!("{text}")); }`, explain why borrowing `text` is rejected, then fix the spawn with `move` and say why the thread must own the value.</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Cloned channel transmitters</t>
+  </si>
+  <si>
+    <t>Write the loop for four workers that all send through one `mpsc` channel: clone `tx` for each worker, move the clone into the closure, then explain why every clone still reaches the same `rx`.</t>
+  </si>
+  <si>
+    <t>`Arc&lt;Mutex&lt;i32&gt;&gt;` shared counter</t>
+  </si>
+  <si>
+    <t>Trace two threads incrementing the same `Arc&lt;Mutex&lt;i32&gt;&gt;` counter and explain how shared ownership is provided and why each update is exclusive.</t>
+  </si>
+  <si>
+    <t>Poisoned mutex lock result</t>
+  </si>
+  <si>
+    <t>For a mutex that was held by a thread when it panicked, write how `lock()` reports the problem and how you would handle the returned result instead of blindly assuming the lock succeeded.</t>
+  </si>
+  <si>
+    <t>Local results then final merge</t>
+  </si>
+  <si>
+    <t>For a word-count task split across four threads, compare one global locked `HashMap` updated for every word with each thread building a local map and merging once at the end. Explain which is better and why.</t>
   </si>
 </sst>
 </file>
@@ -575,7 +611,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -584,6 +620,9 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -604,8 +643,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E64" displayName="RevisionMistakeTracker" name="RevisionMistakeTracker" id="1" totalsRowShown="0">
-  <autoFilter ref="A1:E64"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E69" displayName="RevisionMistakeTracker" name="RevisionMistakeTracker" id="1" totalsRowShown="0">
+  <autoFilter ref="A1:E69"/>
   <tableColumns count="5">
     <tableColumn name="Topic sheet" id="1"/>
     <tableColumn name="Question number" id="2"/>
@@ -905,14 +944,14 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="4" width="28.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="4" width="24.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="4" width="68.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="4" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="28.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="24.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="5" width="68.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="5" width="14.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="24" customFormat="1" s="1">
@@ -1714,7 +1753,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="32.25" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="54" customFormat="1" s="1">
       <c r="A48" s="3" t="s">
         <v>117</v>
       </c>
@@ -1731,7 +1770,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="32.25" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="54" customFormat="1" s="1">
       <c r="A49" s="3" t="s">
         <v>117</v>
       </c>
@@ -1748,7 +1787,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="45.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="54" customFormat="1" s="1">
       <c r="A50" s="3" t="s">
         <v>128</v>
       </c>
@@ -1765,7 +1804,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="32.25" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="54" customFormat="1" s="1">
       <c r="A51" s="3" t="s">
         <v>128</v>
       </c>
@@ -1782,7 +1821,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="45.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="54" customFormat="1" s="1">
       <c r="A52" s="3" t="s">
         <v>128</v>
       </c>
@@ -1931,9 +1970,11 @@
       <c r="D60" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="E60" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="54" customFormat="1" s="1">
+      <c r="E60" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="32.25" customFormat="1" s="1">
       <c r="A61" s="3" t="s">
         <v>152</v>
       </c>
@@ -1950,7 +1991,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="54" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="32.25" customFormat="1" s="1">
       <c r="A62" s="3" t="s">
         <v>152</v>
       </c>
@@ -1963,9 +2004,11 @@
       <c r="D62" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="E62" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="54" customFormat="1" s="1">
+      <c r="E62" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="32.25" customFormat="1" s="1">
       <c r="A63" s="3" t="s">
         <v>159</v>
       </c>
@@ -1978,9 +2021,11 @@
       <c r="D63" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="E63" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="54" customFormat="1" s="1">
+      <c r="E63" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="32.25" customFormat="1" s="1">
       <c r="A64" s="3" t="s">
         <v>159</v>
       </c>
@@ -1993,7 +2038,90 @@
       <c r="D64" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="E64" s="3"/>
+      <c r="E64" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="45.75" customFormat="1" s="1">
+      <c r="A65" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="E65" s="4" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="45.75" customFormat="1" s="1">
+      <c r="A66" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="E66" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="54" customFormat="1" s="1">
+      <c r="A67" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="E67" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="54" customFormat="1" s="1">
+      <c r="A68" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="E68" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="54" customFormat="1" s="1">
+      <c r="A69" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="E69" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add C and Rust study packs for memory debugging tools and custom iterators
- Created a focused revision sheet for C memory debugging tools, including Valgrind and AddressSanitizer, with examples and practice questions.
- Developed a Python script to generate the C memory debugging tools study pack PDF.
- Added a focused revision sheet for Rust custom iterators and pipelines, detailing iterator behavior, common adapters, and practice questions.
- Implemented a Python script to generate the Rust custom iterators and pipelines study pack PDF.
- Updated markdown topic lists to reflect the addition of new study packs.
</commit_message>
<xml_diff>
--- a/revision-mistake-log.xlsx
+++ b/revision-mistake-log.xlsx
@@ -83,8 +83,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RevisionMistakeTracker" displayName="RevisionMistakeTracker" ref="A1:E76" totalsRowShown="0">
-  <autoFilter ref="A1:E76"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RevisionMistakeTracker" displayName="RevisionMistakeTracker" ref="A1:E87" totalsRowShown="0">
+  <autoFilter ref="A1:E87"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Topic sheet"/>
     <tableColumn id="2" name="Question number"/>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="E69" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2047,7 +2047,7 @@
       </c>
       <c r="E72" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="E75" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2154,6 +2154,303 @@
         </is>
       </c>
       <c r="E76" t="inlineStr" s="2">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="54" customHeight="1">
+      <c r="A77" t="inlineStr" s="2">
+        <is>
+          <t>C Memory Debugging Tools</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr" s="2">
+        <is>
+          <t>Use-after-free dereference</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr" s="2">
+        <is>
+          <t>Given `free(p); return *p;`, explain why `p` is stale after `free`, what dereferencing it means, and what kind of behaviour C gives for that access.</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="54" customHeight="1">
+      <c r="A78" t="inlineStr" s="2">
+        <is>
+          <t>C Memory Debugging Tools</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr" s="2">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr" s="2">
+        <is>
+          <t>Valgrind full leak-check command</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr" s="2">
+        <is>
+          <t>Write the command to run `./app` under Valgrind with full leak checking, then add one useful option for tracing where uninitialised values came from.</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="54" customHeight="1">
+      <c r="A79" t="inlineStr" s="2">
+        <is>
+          <t>C Memory Debugging Tools</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr" s="2">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr" s="2">
+        <is>
+          <t>Debug info for memory-tool reports</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr" s="2">
+        <is>
+          <t>Explain what `-g` adds to a debug build and why memory tools give more useful reports when source-level debug information is present.</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="54" customHeight="1">
+      <c r="A80" t="inlineStr" s="2">
+        <is>
+          <t>C Memory Debugging Tools</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr" s="2">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr" s="2">
+        <is>
+          <t>First memory-tool error</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr" s="2">
+        <is>
+          <t>A memory tool prints several invalid reads and writes. Explain which report you would investigate first and why later reports may be consequences of earlier corruption.</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="54" customHeight="1">
+      <c r="A81" t="inlineStr" s="2">
+        <is>
+          <t>C Memory Debugging Tools</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr" s="2">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr" s="2">
+        <is>
+          <t>Memory bugs and undefined behaviour</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr" s="2">
+        <is>
+          <t>A C program prints the expected answer but AddressSanitizer reports an invalid access. Explain why the program is still wrong and connect this to undefined behaviour.</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="54" customHeight="1">
+      <c r="A82" t="inlineStr" s="2">
+        <is>
+          <t>Rust Custom Iterators and Pipelines</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr" s="2">
+        <is>
+          <t>Lazy `map` adapter</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr" s="2">
+        <is>
+          <t>Given `let doubled = values.iter().map(|n| n * 2);`, explain what `doubled` contains before any consumer runs, then show one way to produce actual values.</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="54" customHeight="1">
+      <c r="A83" t="inlineStr" s="2">
+        <is>
+          <t>Rust Custom Iterators and Pipelines</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr" s="2">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr" s="2">
+        <is>
+          <t>Even-square pipeline collection</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr" s="2">
+        <is>
+          <t>Starting with `let values = vec![1, 2, 3, 4];`, write the full iterator chain that filters even numbers, maps them to squares, and collects with an explicit `Vec` type.</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="54" customHeight="1">
+      <c r="A84" t="inlineStr" s="2">
+        <is>
+          <t>Rust Custom Iterators and Pipelines</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr" s="2">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr" s="2">
+        <is>
+          <t>Text word pipeline</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr" s="2">
+        <is>
+          <t>Given `let text = "Rust, rust! C?";`, write a pipeline that splits into words, lowercases each cleaned word, removes empty strings, and collects into `Vec&lt;String&gt;`.</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="54" customHeight="1">
+      <c r="A85" t="inlineStr" s="2">
+        <is>
+          <t>Rust Custom Iterators and Pipelines</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr" s="2">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr" s="2">
+        <is>
+          <t>HashMap score pipeline</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr" s="2">
+        <is>
+          <t>Given a map of team names to scores, collect entries with scores at least 10 into a vector, making clear where filtering and copying out borrowed values happen.</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="54" customHeight="1">
+      <c r="A86" t="inlineStr" s="2">
+        <is>
+          <t>Rust Custom Iterators and Pipelines</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr" s="2">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr" s="2">
+        <is>
+          <t>Custom iterator field access</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr" s="2">
+        <is>
+          <t>In `Counter::next`, fix a body that tries to read `self[current]`; write the correct field access syntax for `current` and explain why indexing syntax is wrong.</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="54" customHeight="1">
+      <c r="A87" t="inlineStr" s="2">
+        <is>
+          <t>Rust Custom Iterators and Pipelines</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr" s="2">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr" s="2">
+        <is>
+          <t>`next` returns `Option`</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr" s="2">
+        <is>
+          <t>For a custom counter iterator, explain both possible `next` results: what is returned when there is another value and what is returned when the iterator is finished.</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr" s="2">
         <is>
           <t/>
         </is>

</xml_diff>

<commit_message>
Add study packs for C control flow, string processing, and C++ multiple inheritance
- Created `make_c_control_flow_problem_solving_study_pack.py` to cover C control flow concepts including conditions, loops, factorials, and compilation processes.
- Created `make_c_string_processing_study_pack.py` to address C string handling, including null terminators, standard library functions, character classification, and in-place editing.
- Created `make_cpp_multiple_inheritance_study_pack.py` to explain C++ multiple inheritance, including access specifiers, the diamond problem, virtual base classes, and runtime dispatch.
</commit_message>
<xml_diff>
--- a/revision-mistake-log.xlsx
+++ b/revision-mistake-log.xlsx
@@ -83,8 +83,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RevisionMistakeTracker" displayName="RevisionMistakeTracker" ref="A1:E87" totalsRowShown="0">
-  <autoFilter ref="A1:E87"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RevisionMistakeTracker" displayName="RevisionMistakeTracker" ref="A1:E102" totalsRowShown="0">
+  <autoFilter ref="A1:E102"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Topic sheet"/>
     <tableColumn id="2" name="Question number"/>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="E65" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="E67" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1993,7 +1993,7 @@
       </c>
       <c r="E70" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="E71" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="E73" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="E74" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="E77" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="E80" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2290,7 +2290,7 @@
       </c>
       <c r="E81" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2317,7 +2317,7 @@
       </c>
       <c r="E82" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2344,7 +2344,7 @@
       </c>
       <c r="E83" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2398,7 +2398,7 @@
       </c>
       <c r="E85" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2425,7 +2425,7 @@
       </c>
       <c r="E86" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2451,6 +2451,411 @@
         </is>
       </c>
       <c r="E87" t="inlineStr" s="2">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="54" customHeight="1">
+      <c r="A88" t="inlineStr" s="2">
+        <is>
+          <t>C Basic Syntax and Program Layout</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr" s="2">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr" s="2">
+        <is>
+          <t>Semicolons after declarations</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr" s="2">
+        <is>
+          <t>Given a short program containing `int x = 4`, `double y = 2.5`, and a `printf` call without statement endings, fix every missing semicolon and explain why the declarations need them.</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr" s="2">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="54" customHeight="1">
+      <c r="A89" t="inlineStr" s="2">
+        <is>
+          <t>C Basic Syntax and Program Layout</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr" s="2">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr" s="2">
+        <is>
+          <t>Tab escape sequence</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr" s="2">
+        <is>
+          <t>Write a `printf` statement that prints two integer values separated by a tab and followed by a newline, using the correct escape sequence for the tab.</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr" s="2">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="54" customHeight="1">
+      <c r="A90" t="inlineStr" s="2">
+        <is>
+          <t>C Basic Syntax and Program Layout</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr" s="2">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr" s="2">
+        <is>
+          <t>`return 0` from `main`</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr" s="2">
+        <is>
+          <t>For a small `int main(void)` program that finishes normally, write the final return statement and explain what status it reports to the operating system.</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="54" customHeight="1">
+      <c r="A91" t="inlineStr" s="2">
+        <is>
+          <t>C Control Flow and Problem Solving</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr" s="2">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr" s="2">
+        <is>
+          <t>Factorial loop variable</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr" s="2">
+        <is>
+          <t>Write a factorial loop that counts down from `n` to `1`, then trace `n = 4` and identify which variable must be multiplied into the accumulator each iteration.</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr" s="2">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="54" customHeight="1">
+      <c r="A92" t="inlineStr" s="2">
+        <is>
+          <t>C Control Flow and Problem Solving</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr" s="2">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr" s="2">
+        <is>
+          <t>`e` approximation loop bounds</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr" s="2">
+        <is>
+          <t>Write an `approximate_e(int terms)` loop using factorial terms, making sure the division is floating-point and the loop produces exactly `terms` terms.</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="54" customHeight="1">
+      <c r="A93" t="inlineStr" s="2">
+        <is>
+          <t>C Control Flow and Problem Solving</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr" s="2">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr" s="2">
+        <is>
+          <t>Object file compile and link workflow</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr" s="2">
+        <is>
+          <t>For a program split across `main.c` and `maths.c`, write the commands that produce `main.o` and `maths.o`, then link them into an executable.</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="54" customHeight="1">
+      <c r="A94" t="inlineStr" s="2">
+        <is>
+          <t>C String Processing</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr" s="2">
+        <is>
+          <t>`sizeof` on char arrays</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr" s="2">
+        <is>
+          <t>For `char s[20] = "Hello world";`, calculate the storage size and visible character count, then explain why the two numbers are different.</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="54" customHeight="1">
+      <c r="A95" t="inlineStr" s="2">
+        <is>
+          <t>C String Processing</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr" s="2">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr" s="2">
+        <is>
+          <t>Null terminator and `sizeof`</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr" s="2">
+        <is>
+          <t>For `char s[20] = "Hello world"; s[0] = '\0';`, calculate `sizeof(s)` and `strlen(s)`, then identify which result changed.</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="54" customHeight="1">
+      <c r="A96" t="inlineStr" s="2">
+        <is>
+          <t>C String Processing</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr" s="2">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr" s="2">
+        <is>
+          <t>In-place normalise write index</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr" s="2">
+        <is>
+          <t>Trace what goes wrong if an in-place normalise loop increments `write` when punctuation is skipped, then write the corrected loop for `"A, B!"` and the required character-function include.</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="54" customHeight="1">
+      <c r="A97" t="inlineStr" s="2">
+        <is>
+          <t>C String Processing</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr" s="2">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr" s="2">
+        <is>
+          <t>Bounded copy loop limit</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr" s="2">
+        <is>
+          <t>For `char dest[5]` copying from `"Hello"`, compare loop guards `i &lt;= len - 1` and `i &lt; len - 1`; choose the safe one and show where the null terminator is written.</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="54" customHeight="1">
+      <c r="A98" t="inlineStr" s="2">
+        <is>
+          <t>C++ Multiple Inheritance</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr" s="2">
+        <is>
+          <t>Protected member access in derived methods</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr" s="2">
+        <is>
+          <t>Given a base class with private `i` and protected `j`, and a derived method containing `i = 0; j = 0;`, mark which assignment compiles and explain the access rule using the derived method context.</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="54" customHeight="1">
+      <c r="A99" t="inlineStr" s="2">
+        <is>
+          <t>C++ Multiple Inheritance</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr" s="2">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr" s="2">
+        <is>
+          <t>Diamond ambiguity is compile-time</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr" s="2">
+        <is>
+          <t>For `Bottom` inheriting from both `Left` and `Right`, where each path contains `Base::value`, decide what happens to `b.value = 10;` and whether the issue is compile-time or runtime.</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="54" customHeight="1">
+      <c r="A100" t="inlineStr" s="2">
+        <is>
+          <t>C++ Multiple Inheritance</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr" s="2">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr" s="2">
+        <is>
+          <t>Selecting one diamond base path</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr" s="2">
+        <is>
+          <t>In a non-virtual diamond with `Bottom b`, write the assignment that sets the `value` reached through `Left` rather than the one reached through `Right`.</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="54" customHeight="1">
+      <c r="A101" t="inlineStr" s="2">
+        <is>
+          <t>C++ Multiple Inheritance</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr" s="2">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr" s="2">
+        <is>
+          <t>Virtual dispatch trace</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr" s="2">
+        <is>
+          <t>Given `Animal::speak` is virtual, `Dog::speak` prints `Bark Fido`, and an `Animal *` points at a `Dog`, trace the call through the base pointer and explain why the dog version runs.</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="54" customHeight="1">
+      <c r="A102" t="inlineStr" s="2">
+        <is>
+          <t>C++ Multiple Inheritance</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr" s="2">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr" s="2">
+        <is>
+          <t>Abstract base class instantiation</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr" s="2">
+        <is>
+          <t>Given `virtual void speak() const = 0;` in `Animal`, decide whether `Animal a("Rex");` compiles, then show what a concrete derived class must provide before it can be instantiated.</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr" s="2">
         <is>
           <t/>
         </is>

</xml_diff>

<commit_message>
Add Rust tooling and Cargo study pack, including key concepts and practice questions
- Introduced a new Python script to generate a PDF study pack for Rust tooling and Cargo.
- Updated existing PDF study packs for custom iterators and pipelines, expressions and statements, ownership and borrowing, and added a new study pack for Rust tooling and Cargo.
- Enhanced clarity and correctness in code examples and explanations throughout the documents.
- Included practice questions and mark schemes for self-assessment in the new Rust tooling and Cargo study pack.
</commit_message>
<xml_diff>
--- a/revision-mistake-log.xlsx
+++ b/revision-mistake-log.xlsx
@@ -83,8 +83,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RevisionMistakeTracker" displayName="RevisionMistakeTracker" ref="A1:E102" totalsRowShown="0">
-  <autoFilter ref="A1:E102"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RevisionMistakeTracker" displayName="RevisionMistakeTracker" ref="A1:E117" totalsRowShown="0">
+  <autoFilter ref="A1:E117"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Topic sheet"/>
     <tableColumn id="2" name="Question number"/>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="E84" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2587,7 +2587,7 @@
       </c>
       <c r="E92" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2614,7 +2614,7 @@
       </c>
       <c r="E93" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2641,7 +2641,7 @@
       </c>
       <c r="E94" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2668,7 +2668,7 @@
       </c>
       <c r="E95" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2695,7 +2695,7 @@
       </c>
       <c r="E96" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2722,7 +2722,7 @@
       </c>
       <c r="E97" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2749,7 +2749,7 @@
       </c>
       <c r="E98" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2776,7 +2776,7 @@
       </c>
       <c r="E99" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="E100" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2830,7 +2830,7 @@
       </c>
       <c r="E101" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2856,6 +2856,411 @@
         </is>
       </c>
       <c r="E102" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="54" customHeight="1">
+      <c r="A103" t="inlineStr" s="2">
+        <is>
+          <t>C++ Classes: Access Control and Header Files</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr" s="2">
+        <is>
+          <t>Complete guarded class header</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr" s="2">
+        <is>
+          <t>A header `counter.h` declares a `Counter` class and may be included through several files. Write the complete guarded header around the class declaration so repeated inclusion is safe.</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="54" customHeight="1">
+      <c r="A104" t="inlineStr" s="2">
+        <is>
+          <t>C++ Classes: Access Control and Header Files</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr" s="2">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr" s="2">
+        <is>
+          <t>Scope resolution for member definitions</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr" s="2">
+        <is>
+          <t>In `counter.cpp`, fix `void increment() { count++; }` so it defines the member declared in `Counter`, then explain what the prefix connects the function body to.</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="54" customHeight="1">
+      <c r="A105" t="inlineStr" s="2">
+        <is>
+          <t>C++ Classes: Access Control and Header Files</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr" s="2">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr" s="2">
+        <is>
+          <t>Balanced include guard</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr" s="2">
+        <is>
+          <t>Complete a guarded `sensor.h` header from the opening conditional directive through the final closing directive, using a sensible guard name.</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="54" customHeight="1">
+      <c r="A106" t="inlineStr" s="2">
+        <is>
+          <t>C++ Classes: Access Control and Header Files</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr" s="2">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr" s="2">
+        <is>
+          <t>Repeated include redefinition fix</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr" s="2">
+        <is>
+          <t>`grandparent.h` defines `struct Data` and is included both directly and through `parent.h`. Wrap `grandparent.h` so `child.cpp` does not see two definitions.</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="54" customHeight="1">
+      <c r="A107" t="inlineStr" s="2">
+        <is>
+          <t>C++ Classes: Access Control and Header Files</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr" s="2">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr" s="2">
+        <is>
+          <t>Destructor for owned array</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr" s="2">
+        <is>
+          <t>Given `class Buffer { char *data; public: Buffer(int size) { data = new char[size]; } };`, add the destructor and explain why a default destructor is not enough.</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="54" customHeight="1">
+      <c r="A108" t="inlineStr" s="2">
+        <is>
+          <t>C++ Classes: Access Control and Header Files</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr" s="2">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr" s="2">
+        <is>
+          <t>`new`/`delete` vs `malloc`/`free` for objects</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr" s="2">
+        <is>
+          <t>For a class with a constructor and destructor, compare allocation with `new` and `malloc`, then compare cleanup with `delete` and `free`; say which operations run object lifetime code.</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="54" customHeight="1">
+      <c r="A109" t="inlineStr" s="2">
+        <is>
+          <t>C Struct Exercises: Points and Rectangles</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr" s="2">
+        <is>
+          <t>Semicolons in struct field declarations</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr" s="2">
+        <is>
+          <t>Repair `typedef struct { double x double y } Point;` so it is a valid C type definition, then declare one `Point` variable.</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="54" customHeight="1">
+      <c r="A110" t="inlineStr" s="2">
+        <is>
+          <t>C Struct Exercises: Points and Rectangles</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr" s="2">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr" s="2">
+        <is>
+          <t>Nested struct field semicolons</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr" s="2">
+        <is>
+          <t>Write a `Rectangle` type containing `Point bottom_left` and `Point top_right`, making sure the field declarations and the whole type definition are correctly terminated.</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="54" customHeight="1">
+      <c r="A111" t="inlineStr" s="2">
+        <is>
+          <t>C Struct Exercises: Points and Rectangles</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr" s="2">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr" s="2">
+        <is>
+          <t>Updating caller-owned struct through pointer</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr" s="2">
+        <is>
+          <t>Fix `void move_point(Point p, double dx, double dy)` so the caller's point is changed, then show the corrected call for a variable named `pt`.</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="54" customHeight="1">
+      <c r="A112" t="inlineStr" s="2">
+        <is>
+          <t>C Struct Exercises: Points and Rectangles</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr" s="2">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr" s="2">
+        <is>
+          <t>Choosing pass-by-value for structs</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr" s="2">
+        <is>
+          <t>A function only reads a small `Point` to calculate a result and must not modify the caller's value. Choose a by-value or pointer parameter and justify the choice.</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="54" customHeight="1">
+      <c r="A113" t="inlineStr" s="2">
+        <is>
+          <t>C Struct Exercises: Points and Rectangles</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr" s="2">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr" s="2">
+        <is>
+          <t>Struct size, padding, and alignment</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr" s="2">
+        <is>
+          <t>Compare `sizeof` for a two-double `Point` with a struct containing `char c; double x;`. Explain why the mixed-field struct may be larger than the simple sum of field sizes.</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="54" customHeight="1">
+      <c r="A114" t="inlineStr" s="2">
+        <is>
+          <t>Rust Tooling and Cargo</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr" s="2">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr" s="2">
+        <is>
+          <t>Cargo as build tool and package manager</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr" s="2">
+        <is>
+          <t>A Rust project uses Cargo where a C project might need separate build and dependency tools. Name the two jobs Cargo handles and give one command or file connected to each job.</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="54" customHeight="1">
+      <c r="A115" t="inlineStr" s="2">
+        <is>
+          <t>Rust Tooling and Cargo</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr" s="2">
+        <is>
+          <t>`cargo new` project layout</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr" s="2">
+        <is>
+          <t>After running `cargo new hello_rust`, list the generated source entry point path and the main Cargo config files, then say which file contains the starting `main` function.</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="54" customHeight="1">
+      <c r="A116" t="inlineStr" s="2">
+        <is>
+          <t>Rust Tooling and Cargo</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr" s="2">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr" s="2">
+        <is>
+          <t>`cargo run` with unchanged source</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr" s="2">
+        <is>
+          <t>After a successful build, no source files have changed. Explain what `cargo run` does next and whether it recompiles or runs the existing binary.</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="54" customHeight="1">
+      <c r="A117" t="inlineStr" s="2">
+        <is>
+          <t>Rust Tooling and Cargo</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr" s="2">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr" s="2">
+        <is>
+          <t>Opening Rust Book offline</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr" s="2">
+        <is>
+          <t>On a machine with Rust docs installed but no internet connection, write the command that opens the Rust Book and distinguish it from opening the general local Rust documentation.</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr" s="2">
         <is>
           <t/>
         </is>

</xml_diff>

<commit_message>
Add ECM2433 Mock Exam Paper 2 Generation Script
- Created a new Python script `make_ecm2433_mock_exam_2.py` to generate a mock exam paper in PDF format.
- Implemented styles for various sections of the exam paper using ReportLab.
- Added structured questions and answers covering topics such as C, C++, Rust, and Makefile.
- Included guidelines and formatting for the exam paper layout.
- Added answers and marking notes at the end of the document for reference.
- Updated revision-correct-rules.md with new questions and answers related to Makefile, heap allocation, sorting, exception handling, and more.
- Updated revision-mistake-log.xlsx to reflect changes in the revision log.
</commit_message>
<xml_diff>
--- a/revision-mistake-log.xlsx
+++ b/revision-mistake-log.xlsx
@@ -83,8 +83,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RevisionMistakeTracker" displayName="RevisionMistakeTracker" ref="A1:E142" totalsRowShown="0">
-  <autoFilter ref="A1:E142"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RevisionMistakeTracker" displayName="RevisionMistakeTracker" ref="A1:E155" totalsRowShown="0">
+  <autoFilter ref="A1:E155"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Topic sheet"/>
     <tableColumn id="2" name="Question number"/>
@@ -3532,7 +3532,7 @@
       </c>
       <c r="E127" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="E132" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3694,7 +3694,7 @@
       </c>
       <c r="E133" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3721,7 +3721,7 @@
       </c>
       <c r="E134" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3775,7 +3775,7 @@
       </c>
       <c r="E136" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3829,7 +3829,7 @@
       </c>
       <c r="E138" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="E139" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3883,7 +3883,7 @@
       </c>
       <c r="E140" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3910,7 +3910,7 @@
       </c>
       <c r="E141" t="inlineStr" s="2">
         <is>
-          <t/>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3936,6 +3936,357 @@
         </is>
       </c>
       <c r="E142" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="54" customHeight="1">
+      <c r="A143" t="inlineStr" s="2">
+        <is>
+          <t>ECM2433 Mock Paper 1</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr" s="2">
+        <is>
+          <t>1b</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr" s="2">
+        <is>
+          <t>Makefile clean rule</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr" s="2">
+        <is>
+          <t>For the mock project with `main.c`, `stats.c`, and `stats.h`, write the full Makefile fragment for `report`, then include the `clean` recipe that removes all object files and the `report` executable.</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="54" customHeight="1">
+      <c r="A144" t="inlineStr" s="2">
+        <is>
+          <t>ECM2433 Mock Paper 1</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr" s="2">
+        <is>
+          <t>1c</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr" s="2">
+        <is>
+          <t>Heap string copy allocation</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr" s="2">
+        <is>
+          <t>In the `copy_label(const char *src)` stub, fill in `char *copy = ...`, the allocation failure check, and the copy step so the result includes room for the string terminator.</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="54" customHeight="1">
+      <c r="A145" t="inlineStr" s="2">
+        <is>
+          <t>ECM2433 Mock Paper 1</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr" s="2">
+        <is>
+          <t>1d</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr" s="2">
+        <is>
+          <t>`qsort` comparator ordering</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr" s="2">
+        <is>
+          <t>For `typedef struct { char name[16]; int score; } Entry;`, complete `compare_entries` and `sort_entries` so `qsort` orders score descending and name ascending on ties.</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="54" customHeight="1">
+      <c r="A146" t="inlineStr" s="2">
+        <is>
+          <t>ECM2433 Mock Paper 1</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr" s="2">
+        <is>
+          <t>1e</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr" s="2">
+        <is>
+          <t>Dangling pointer after `free`</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr" s="2">
+        <is>
+          <t>For the mock code `int *p = malloc(sizeof *p); *p = 10; free(p); printf("%d\n", *p);`, explain why `p` is dangling and what C behaviour dereferencing it gives.</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="54" customHeight="1">
+      <c r="A147" t="inlineStr" s="2">
+        <is>
+          <t>ECM2433 Mock Paper 1</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr" s="2">
+        <is>
+          <t>2b</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr" s="2">
+        <is>
+          <t>Rule of three for raw heap arrays</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr" s="2">
+        <is>
+          <t>For the mock `Buffer` class with `char *data`, `new char[size]`, and `~Buffer() = default`, identify the leak and explain why a raw-owning fix also needs a copy constructor and copy assignment operator.</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="54" customHeight="1">
+      <c r="A148" t="inlineStr" s="2">
+        <is>
+          <t>ECM2433 Mock Paper 1</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr" s="2">
+        <is>
+          <t>2d</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr" s="2">
+        <is>
+          <t>`shared_ptr` last owner lifetime</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr" s="2">
+        <is>
+          <t>Trace the mock `shared_ptr`/`weak_ptr` code with `a`, `watch`, `b = a`, and `a.reset()`: decide whether `watch.lock()` succeeds and when the shared int is destroyed.</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="54" customHeight="1">
+      <c r="A149" t="inlineStr" s="2">
+        <is>
+          <t>ECM2433 Mock Paper 1</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr" s="2">
+        <is>
+          <t>2e</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr" s="2">
+        <is>
+          <t>Catching exceptions by const reference</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr" s="2">
+        <is>
+          <t>For `catch (const std::invalid_argument&amp; error)` after throwing `std::invalid_argument("negative age")`, explain why const reference is used and what `error.what()` prints.</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="54" customHeight="1">
+      <c r="A150" t="inlineStr" s="2">
+        <is>
+          <t>ECM2433 Mock Paper 1</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr" s="2">
+        <is>
+          <t>3d</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr" s="2">
+        <is>
+          <t>Float sorting unwrap after `partial_cmp`</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr" s="2">
+        <is>
+          <t>Given `let mut readings = vec![(0.5, 2), (0.1, 9), (0.5, 1)];`, write the `sort_by` call for float ascending and id descending, including `partial_cmp(...).unwrap()`.</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="54" customHeight="1">
+      <c r="A151" t="inlineStr" s="2">
+        <is>
+          <t>ECM2433 Mock Paper 1</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr" s="2">
+        <is>
+          <t>3e</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr" s="2">
+        <is>
+          <t>Semicolon after Rust `let` parse statement</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr" s="2">
+        <is>
+          <t>In the mock `parse_count` function returning `Result&lt;i32, ParseIntError&gt;`, write the parsing `let n = ...?;` line and explain why that line needs a semicolon but `Ok(n)` does not.</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="54" customHeight="1">
+      <c r="A152" t="inlineStr" s="2">
+        <is>
+          <t>ECM2433 Mock Paper 1</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr" s="2">
+        <is>
+          <t>4a</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr" s="2">
+        <is>
+          <t>Channel send and dropping original sender</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr" s="2">
+        <is>
+          <t>In the mock `mpsc` program with `let (tx, rx) = mpsc::channel()` and `for id in 0..4`, spawn workers that send `id * 10`, then explain why `drop(tx)` is needed before `for value in rx` can finish.</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="54" customHeight="1">
+      <c r="A153" t="inlineStr" s="2">
+        <is>
+          <t>ECM2433 Mock Paper 1</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr" s="2">
+        <is>
+          <t>4b</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr" s="2">
+        <is>
+          <t>Mutex lock result and guard lifetime</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr" s="2">
+        <is>
+          <t>In the mock `Arc&lt;Mutex&lt;i32&gt;&gt;` counter loop, complete the spawned closure so it locks, unwraps, increments through the guard, and explain when the guard unlocks the mutex.</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="54" customHeight="1">
+      <c r="A154" t="inlineStr" s="2">
+        <is>
+          <t>ECM2433 Mock Paper 1</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr" s="2">
+        <is>
+          <t>4c</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr" s="2">
+        <is>
+          <t>Generic bounds for compare and display</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr" s="2">
+        <is>
+          <t>For the mock `show_larger&lt;T&gt;` body using `if a &gt; b` and `println!("{winner}")`, fix the generic signature and name the trait bounds needed for those two operations.</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="54" customHeight="1">
+      <c r="A155" t="inlineStr" s="2">
+        <is>
+          <t>ECM2433 Mock Paper 1</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr" s="2">
+        <is>
+          <t>4d</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr" s="2">
+        <is>
+          <t>Boxed recursive enum size</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr" s="2">
+        <is>
+          <t>For the mock enum `List { Cons(i32, List), Nil }`, replace the recursive field with `Box&lt;List&gt;` and explain why the boxed pointer gives the enum a known size.</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr" s="2">
         <is>
           <t/>
         </is>

</xml_diff>

<commit_message>
Update README and add mock exam mistakes documentation; separate mock exam mistakes into their own file
</commit_message>
<xml_diff>
--- a/revision-mistake-log.xlsx
+++ b/revision-mistake-log.xlsx
@@ -83,8 +83,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RevisionMistakeTracker" displayName="RevisionMistakeTracker" ref="A1:E155" totalsRowShown="0">
-  <autoFilter ref="A1:E155"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RevisionMistakeTracker" displayName="RevisionMistakeTracker" ref="A1:E142" totalsRowShown="0">
+  <autoFilter ref="A1:E142"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Topic sheet"/>
     <tableColumn id="2" name="Question number"/>
@@ -3941,357 +3941,6 @@
         </is>
       </c>
     </row>
-    <row r="143" ht="54" customHeight="1">
-      <c r="A143" t="inlineStr" s="2">
-        <is>
-          <t>ECM2433 Mock Paper 1</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr" s="2">
-        <is>
-          <t>1b</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr" s="2">
-        <is>
-          <t>Makefile clean rule</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr" s="2">
-        <is>
-          <t>For the mock project with `main.c`, `stats.c`, and `stats.h`, write the full Makefile fragment for `report`, then include the `clean` recipe that removes all object files and the `report` executable.</t>
-        </is>
-      </c>
-      <c r="E143" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="144" ht="54" customHeight="1">
-      <c r="A144" t="inlineStr" s="2">
-        <is>
-          <t>ECM2433 Mock Paper 1</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr" s="2">
-        <is>
-          <t>1c</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr" s="2">
-        <is>
-          <t>Heap string copy allocation</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr" s="2">
-        <is>
-          <t>In the `copy_label(const char *src)` stub, fill in `char *copy = ...`, the allocation failure check, and the copy step so the result includes room for the string terminator.</t>
-        </is>
-      </c>
-      <c r="E144" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="145" ht="54" customHeight="1">
-      <c r="A145" t="inlineStr" s="2">
-        <is>
-          <t>ECM2433 Mock Paper 1</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr" s="2">
-        <is>
-          <t>1d</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr" s="2">
-        <is>
-          <t>`qsort` comparator ordering</t>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr" s="2">
-        <is>
-          <t>For `typedef struct { char name[16]; int score; } Entry;`, complete `compare_entries` and `sort_entries` so `qsort` orders score descending and name ascending on ties.</t>
-        </is>
-      </c>
-      <c r="E145" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="146" ht="54" customHeight="1">
-      <c r="A146" t="inlineStr" s="2">
-        <is>
-          <t>ECM2433 Mock Paper 1</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr" s="2">
-        <is>
-          <t>1e</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr" s="2">
-        <is>
-          <t>Dangling pointer after `free`</t>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr" s="2">
-        <is>
-          <t>For the mock code `int *p = malloc(sizeof *p); *p = 10; free(p); printf("%d\n", *p);`, explain why `p` is dangling and what C behaviour dereferencing it gives.</t>
-        </is>
-      </c>
-      <c r="E146" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="147" ht="54" customHeight="1">
-      <c r="A147" t="inlineStr" s="2">
-        <is>
-          <t>ECM2433 Mock Paper 1</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr" s="2">
-        <is>
-          <t>2b</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr" s="2">
-        <is>
-          <t>Rule of three for raw heap arrays</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr" s="2">
-        <is>
-          <t>For the mock `Buffer` class with `char *data`, `new char[size]`, and `~Buffer() = default`, identify the leak and explain why a raw-owning fix also needs a copy constructor and copy assignment operator.</t>
-        </is>
-      </c>
-      <c r="E147" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="148" ht="54" customHeight="1">
-      <c r="A148" t="inlineStr" s="2">
-        <is>
-          <t>ECM2433 Mock Paper 1</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr" s="2">
-        <is>
-          <t>2d</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr" s="2">
-        <is>
-          <t>`shared_ptr` last owner lifetime</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr" s="2">
-        <is>
-          <t>Trace the mock `shared_ptr`/`weak_ptr` code with `a`, `watch`, `b = a`, and `a.reset()`: decide whether `watch.lock()` succeeds and when the shared int is destroyed.</t>
-        </is>
-      </c>
-      <c r="E148" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="149" ht="54" customHeight="1">
-      <c r="A149" t="inlineStr" s="2">
-        <is>
-          <t>ECM2433 Mock Paper 1</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr" s="2">
-        <is>
-          <t>2e</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr" s="2">
-        <is>
-          <t>Catching exceptions by const reference</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr" s="2">
-        <is>
-          <t>For `catch (const std::invalid_argument&amp; error)` after throwing `std::invalid_argument("negative age")`, explain why const reference is used and what `error.what()` prints.</t>
-        </is>
-      </c>
-      <c r="E149" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="150" ht="54" customHeight="1">
-      <c r="A150" t="inlineStr" s="2">
-        <is>
-          <t>ECM2433 Mock Paper 1</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr" s="2">
-        <is>
-          <t>3d</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr" s="2">
-        <is>
-          <t>Float sorting unwrap after `partial_cmp`</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr" s="2">
-        <is>
-          <t>Given `let mut readings = vec![(0.5, 2), (0.1, 9), (0.5, 1)];`, write the `sort_by` call for float ascending and id descending, including `partial_cmp(...).unwrap()`.</t>
-        </is>
-      </c>
-      <c r="E150" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="151" ht="54" customHeight="1">
-      <c r="A151" t="inlineStr" s="2">
-        <is>
-          <t>ECM2433 Mock Paper 1</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr" s="2">
-        <is>
-          <t>3e</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr" s="2">
-        <is>
-          <t>Semicolon after Rust `let` parse statement</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr" s="2">
-        <is>
-          <t>In the mock `parse_count` function returning `Result&lt;i32, ParseIntError&gt;`, write the parsing `let n = ...?;` line and explain why that line needs a semicolon but `Ok(n)` does not.</t>
-        </is>
-      </c>
-      <c r="E151" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="152" ht="54" customHeight="1">
-      <c r="A152" t="inlineStr" s="2">
-        <is>
-          <t>ECM2433 Mock Paper 1</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr" s="2">
-        <is>
-          <t>4a</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr" s="2">
-        <is>
-          <t>Channel send and dropping original sender</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr" s="2">
-        <is>
-          <t>In the mock `mpsc` program with `let (tx, rx) = mpsc::channel()` and `for id in 0..4`, spawn workers that send `id * 10`, then explain why `drop(tx)` is needed before `for value in rx` can finish.</t>
-        </is>
-      </c>
-      <c r="E152" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="153" ht="54" customHeight="1">
-      <c r="A153" t="inlineStr" s="2">
-        <is>
-          <t>ECM2433 Mock Paper 1</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr" s="2">
-        <is>
-          <t>4b</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr" s="2">
-        <is>
-          <t>Mutex lock result and guard lifetime</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr" s="2">
-        <is>
-          <t>In the mock `Arc&lt;Mutex&lt;i32&gt;&gt;` counter loop, complete the spawned closure so it locks, unwraps, increments through the guard, and explain when the guard unlocks the mutex.</t>
-        </is>
-      </c>
-      <c r="E153" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="154" ht="54" customHeight="1">
-      <c r="A154" t="inlineStr" s="2">
-        <is>
-          <t>ECM2433 Mock Paper 1</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr" s="2">
-        <is>
-          <t>4c</t>
-        </is>
-      </c>
-      <c r="C154" t="inlineStr" s="2">
-        <is>
-          <t>Generic bounds for compare and display</t>
-        </is>
-      </c>
-      <c r="D154" t="inlineStr" s="2">
-        <is>
-          <t>For the mock `show_larger&lt;T&gt;` body using `if a &gt; b` and `println!("{winner}")`, fix the generic signature and name the trait bounds needed for those two operations.</t>
-        </is>
-      </c>
-      <c r="E154" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="155" ht="54" customHeight="1">
-      <c r="A155" t="inlineStr" s="2">
-        <is>
-          <t>ECM2433 Mock Paper 1</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr" s="2">
-        <is>
-          <t>4d</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr" s="2">
-        <is>
-          <t>Boxed recursive enum size</t>
-        </is>
-      </c>
-      <c r="D155" t="inlineStr" s="2">
-        <is>
-          <t>For the mock enum `List { Cons(i32, List), Nil }`, replace the recursive field with `Box&lt;List&gt;` and explain why the boxed pointer gives the enum a known size.</t>
-        </is>
-      </c>
-      <c r="E155" t="inlineStr" s="2">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>